<commit_message>
updated columns of clean data
</commit_message>
<xml_diff>
--- a/1_Data/Amodeo_2024_CABN/Codebook_Amodeo_2024_CABN_Exp1_Clean.xlsx
+++ b/1_Data/Amodeo_2024_CABN/Codebook_Amodeo_2024_CABN_Exp1_Clean.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,26 +413,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Variable_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Variable_description</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Variable_value</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Variable_category</t>
         </is>
@@ -563,17 +551,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Matching</t>
+          <t>Task</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Type of matching task for the trial; indicates whether the shape and label match or not</t>
+          <t>Task type: the kind of shape-label matching task performed in the trial (default self-matching; other tasks e.g. facialExpression-matching, monetaryValue-matching, self-pseudoWords)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Matching;Nonmatching</t>
+          <t>self-matching</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -585,17 +573,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Label_Origin_Identity</t>
+          <t>Matching</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Original identity associated with the label</t>
+          <t>Type of matching task for the trial; indicates whether the shape and label match or not</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Vreemde;Ikzelf;Bekende</t>
+          <t>Matching;Nonmatching</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -607,17 +595,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Label_English_Identity</t>
+          <t>Label_Origin_Identity</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>English translation of the label's identity</t>
+          <t>Original identity associated with the label</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Stranger;Self;Friend</t>
+          <t>Vreemde;Ikzelf;Bekende</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -629,12 +617,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Label_Standardized_Identity</t>
+          <t>Label_English_Identity</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Standardized identity for the label used across experiments</t>
+          <t>English translation of the label's identity</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -651,12 +639,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Shape_Origin_Identity</t>
+          <t>Label_Standardized_Identity</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Original identity associated with the shape stimulus</t>
+          <t>Standardized identity for the label used across experiments</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -673,12 +661,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shape_English_Identity</t>
+          <t>Shape_Origin_Identity</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>English translation of the shape's identity</t>
+          <t>Original identity associated with the shape stimulus</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -695,17 +683,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shape_Standardized_Identity</t>
+          <t>Shape_English_Identity</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Standardized identity for the shape used across experiments</t>
+          <t>English translation of the shape's identity</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Stranger;Self;Close</t>
+          <t>Stranger;Self;Friend</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -717,17 +705,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Response</t>
+          <t>Shape_Standardized_Identity</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Participant's response in the trial</t>
+          <t>Standardized identity for the shape used across experiments</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>n;m</t>
+          <t>Stranger;Self;Close</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -739,34 +727,34 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RT_ms</t>
+          <t>Response</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Reaction time for the response, measured in milliseconds</t>
+          <t>Participant's response in the trial</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>n;m</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Numerical</t>
+          <t>Categorical</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RT_sec</t>
+          <t>RT_ms</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Reaction time for the response, measured in seconds</t>
+          <t>Reaction time for the response, measured in milliseconds</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -783,20 +771,42 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>RT_sec</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Reaction time for the response, measured in seconds</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Numerical</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>ACC</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Accuracy of the participant's response</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>0;1</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Categorical</t>
         </is>

</xml_diff>

<commit_message>
revised column names and order, a major update, many errors might be introduced
</commit_message>
<xml_diff>
--- a/1_Data/Amodeo_2024_CABN/Codebook_Amodeo_2024_CABN_Exp1_Clean.xlsx
+++ b/1_Data/Amodeo_2024_CABN/Codebook_Amodeo_2024_CABN_Exp1_Clean.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,34 +463,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Block</t>
+          <t>Task</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Block number in the experiment; each block may contain practice or experimental trials</t>
+          <t>Task type: the kind of shape-label matching task performed in the trial (default self-matching; other tasks e.g. facialExpression-matching, monetaryValue-matching, self-pseudoWords)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>self-matching</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Numerical</t>
+          <t>Categorical</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Trial</t>
+          <t>Block</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Trial number within the block</t>
+          <t>Block number in the experiment; each block may contain practice or experimental trials</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -507,39 +507,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shape</t>
+          <t>Trial</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Visual shape stimulus presented in the trial</t>
+          <t>Trial number within the block</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>T.bmp;S.bmp;C.bmp</t>
+          <t>Number</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Categorical</t>
+          <t>Numerical</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Label</t>
+          <t>Matching</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Text label presented for matching with the shape</t>
+          <t>Type of matching task for the trial; indicates whether the shape and label match or not</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Vreemde;Ikzelf;Bekende</t>
+          <t>Matching;Nonmatching</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -551,17 +551,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Task</t>
+          <t>Shape</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Task type: the kind of shape-label matching task performed in the trial (default self-matching; other tasks e.g. facialExpression-matching, monetaryValue-matching, self-pseudoWords)</t>
+          <t>Visual shape stimulus presented in the trial</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>self-matching</t>
+          <t>T.bmp;S.bmp;C.bmp</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -573,17 +573,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Matching</t>
+          <t>Shape_Origin_Identity</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Type of matching task for the trial; indicates whether the shape and label match or not</t>
+          <t>Original identity associated with the shape stimulus</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Matching;Nonmatching</t>
+          <t>Stranger;Self;Friend</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -595,17 +595,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Label_Origin_Identity</t>
+          <t>Shape_English_Identity</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Original identity associated with the label</t>
+          <t>English translation of the shape's identity</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vreemde;Ikzelf;Bekende</t>
+          <t>Stranger;Self;Friend</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -617,17 +617,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Label_English_Identity</t>
+          <t>Shape_Standardized_Identity</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>English translation of the label's identity</t>
+          <t>Standardized identity for the shape used across experiments</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Stranger;Self;Friend</t>
+          <t>Stranger;Self;Close</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -639,17 +639,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Label_Standardized_Identity</t>
+          <t>Label</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Standardized identity for the label used across experiments</t>
+          <t>Text label presented for matching with the shape</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Stranger;Self;Friend</t>
+          <t>Vreemde;Ikzelf;Bekende</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -661,17 +661,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shape_Origin_Identity</t>
+          <t>Label_Origin_Identity</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Original identity associated with the shape stimulus</t>
+          <t>Original identity associated with the label</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Stranger;Self;Friend</t>
+          <t>Vreemde;Ikzelf;Bekende</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -683,12 +683,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shape_English_Identity</t>
+          <t>Label_English_Identity</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>English translation of the shape's identity</t>
+          <t>English translation of the label's identity</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -705,17 +705,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shape_Standardized_Identity</t>
+          <t>Label_Standardized_Identity</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Standardized identity for the shape used across experiments</t>
+          <t>Standardized identity for the label used across experiments</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Stranger;Self;Close</t>
+          <t>Stranger;Self;Friend</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -727,17 +727,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Response</t>
+          <t>CorrResponse</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Participant's response in the trial</t>
+          <t>Correct response key for the trial (as designed; from raw CRESP/CorrectAnswer)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>n;m</t>
+          <t>See per-study key mapping</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -749,34 +749,34 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RT_ms</t>
+          <t>Response</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Reaction time for the response, measured in milliseconds</t>
+          <t>Participant's response in the trial</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>n;m</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Numerical</t>
+          <t>Categorical</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RT_sec</t>
+          <t>RT_ms</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Reaction time for the response, measured in seconds</t>
+          <t>Reaction time for the response, measured in milliseconds</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -793,20 +793,42 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>RT_sec</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Reaction time for the response, measured in seconds</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Numerical</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>ACC</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Accuracy of the participant's response</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>0;1</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Categorical</t>
         </is>

</xml_diff>